<commit_message>
Daily NSE scan: 2026-09-17
</commit_message>
<xml_diff>
--- a/output/2026-09-17/enriched_analysis.xlsx
+++ b/output/2026-09-17/enriched_analysis.xlsx
@@ -813,10 +813,10 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>3.681</v>
+        <v>3.694</v>
       </c>
       <c r="Q2" t="n">
-        <v>2877</v>
+        <v>2867</v>
       </c>
       <c r="R2" t="n">
         <v>22.5</v>
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.082</v>
       </c>
       <c r="Q3" t="n">
-        <v>2535</v>
+        <v>2587</v>
       </c>
       <c r="R3" t="n">
-        <v>8.710000000000001</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="S3" t="n">
         <v>36</v>
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.925</v>
+        <v>0.898</v>
       </c>
       <c r="Q4" t="n">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="R4" t="n">
-        <v>8.5</v>
+        <v>8.76</v>
       </c>
       <c r="S4" t="n">
         <v>17</v>
@@ -1359,13 +1359,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.14</v>
+        <v>0.137</v>
       </c>
       <c r="Q5" t="n">
-        <v>2235</v>
+        <v>2298</v>
       </c>
       <c r="R5" t="n">
-        <v>19.6</v>
+        <v>20.1</v>
       </c>
       <c r="S5" t="n">
         <v>-3</v>
@@ -1541,13 +1541,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q6" t="n">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="R6" t="n">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="S6" t="n">
         <v>22</v>
@@ -1723,13 +1723,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.062</v>
+        <v>0.059</v>
       </c>
       <c r="Q7" t="n">
-        <v>1325</v>
+        <v>1394</v>
       </c>
       <c r="R7" t="n">
-        <v>17.8</v>
+        <v>18.8</v>
       </c>
       <c r="S7" t="n">
         <v>55</v>
@@ -1905,10 +1905,10 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.734</v>
+        <v>0.745</v>
       </c>
       <c r="Q8" t="n">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
@@ -2088,10 +2088,10 @@
         <v>0.013</v>
       </c>
       <c r="Q9" t="n">
-        <v>16222</v>
+        <v>16422</v>
       </c>
       <c r="R9" t="n">
-        <v>20.6</v>
+        <v>20.8</v>
       </c>
       <c r="S9" t="n">
         <v>16</v>
@@ -2215,12 +2215,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ALEMBICLTD</t>
+          <t>DIAMONDYD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alembic Limited</t>
+          <t>Prataap Snacks Limited</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -2232,121 +2232,121 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F10" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G10" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I10" t="n">
-        <v>98.95</v>
+        <v>1102.2</v>
       </c>
       <c r="J10" t="n">
-        <v>91.7</v>
+        <v>1173.96</v>
       </c>
       <c r="K10" t="n">
-        <v>7.9</v>
+        <v>-6.1</v>
       </c>
       <c r="L10" t="n">
-        <v>70.88</v>
+        <v>69.75</v>
       </c>
       <c r="M10" t="n">
-        <v>8.49</v>
+        <v>59.58</v>
       </c>
       <c r="N10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>07-08-2026</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.334</v>
+        <v>2.255</v>
       </c>
       <c r="Q10" t="n">
-        <v>2541</v>
+        <v>2642</v>
       </c>
       <c r="R10" t="n">
-        <v>20.8</v>
+        <v>207</v>
       </c>
       <c r="S10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T10" t="n">
-        <v>14</v>
+        <v>19.05</v>
       </c>
       <c r="U10" t="n">
-        <v>-14</v>
+        <v>194</v>
       </c>
       <c r="V10" t="n">
-        <v>0.57</v>
+        <v>1.03</v>
       </c>
       <c r="W10" t="n">
-        <v>16.9</v>
+        <v>3.17</v>
       </c>
       <c r="X10" t="n">
-        <v>0.01</v>
+        <v>0.06</v>
       </c>
       <c r="Y10" t="b">
         <v>1</v>
       </c>
       <c r="Z10" t="n">
-        <v>30</v>
+        <v>3.87</v>
       </c>
       <c r="AA10" t="n">
-        <v>93.37</v>
+        <v>1160.09</v>
       </c>
       <c r="AB10" t="n">
-        <v>92.28</v>
+        <v>1089.12</v>
       </c>
       <c r="AC10" t="n">
-        <v>19.3</v>
+        <v>15.3</v>
       </c>
       <c r="AD10" t="n">
-        <v>91.7739742726077</v>
+        <v>1173.964532439025</v>
       </c>
       <c r="AE10" t="n">
-        <v>7.8</v>
+        <v>-6.1</v>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>07-08-2026</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="AL10" t="n">
-        <v>31</v>
+        <v>84</v>
       </c>
       <c r="AM10" t="n">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="AN10" t="n">
         <v>0</v>
@@ -2355,13 +2355,13 @@
         <v>0</v>
       </c>
       <c r="AP10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AQ10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AR10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AS10" t="n">
         <v>0</v>
@@ -2370,19 +2370,19 @@
         <v>0</v>
       </c>
       <c r="AU10" t="n">
-        <v>45956128</v>
+        <v>0</v>
       </c>
       <c r="AV10" t="n">
-        <v>85826103</v>
+        <v>586966134</v>
       </c>
       <c r="AW10" t="n">
-        <v>85826103</v>
+        <v>595794044</v>
       </c>
       <c r="AX10" t="n">
         <v>0</v>
       </c>
       <c r="AY10" t="n">
-        <v>45956128</v>
+        <v>0</v>
       </c>
       <c r="AZ10" t="n">
         <v>1</v>
@@ -2397,16 +2397,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DIAMONDYD</t>
+          <t>OBCL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Prataap Snacks Limited</t>
+          <t>OBCL LIMITED</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -2414,157 +2414,155 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F11" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G11" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="H11" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="I11" t="n">
-        <v>1102.2</v>
+        <v>56.98</v>
       </c>
       <c r="J11" t="n">
-        <v>1173.96</v>
+        <v>53.45</v>
       </c>
       <c r="K11" t="n">
-        <v>-6.1</v>
+        <v>6.6</v>
       </c>
       <c r="L11" t="n">
-        <v>69.75</v>
+        <v>67.23</v>
       </c>
       <c r="M11" t="n">
-        <v>59.58</v>
+        <v>1.95</v>
       </c>
       <c r="N11" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>07-08-2026</t>
+          <t>15-09-2026</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>2.259</v>
+        <v>1.598</v>
       </c>
       <c r="Q11" t="n">
-        <v>2638</v>
-      </c>
-      <c r="R11" t="n">
-        <v>207</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="R11" t="inlineStr"/>
       <c r="S11" t="n">
         <v>6</v>
       </c>
       <c r="T11" t="n">
-        <v>19.05</v>
+        <v>2.47</v>
       </c>
       <c r="U11" t="n">
-        <v>194</v>
+        <v>-3779</v>
       </c>
       <c r="V11" t="n">
-        <v>1.03</v>
+        <v>-0.05</v>
       </c>
       <c r="W11" t="n">
-        <v>3.17</v>
+        <v>-1.26</v>
       </c>
       <c r="X11" t="n">
-        <v>0.06</v>
+        <v>0.8</v>
       </c>
       <c r="Y11" t="b">
         <v>1</v>
       </c>
       <c r="Z11" t="n">
-        <v>3.87</v>
+        <v>3</v>
       </c>
       <c r="AA11" t="n">
-        <v>1160.09</v>
+        <v>54.13</v>
       </c>
       <c r="AB11" t="n">
-        <v>1089.12</v>
+        <v>55.15</v>
       </c>
       <c r="AC11" t="n">
-        <v>15.3</v>
+        <v>2.5</v>
       </c>
       <c r="AD11" t="n">
-        <v>1173.964532439025</v>
+        <v>53.44741172107844</v>
       </c>
       <c r="AE11" t="n">
-        <v>-6.1</v>
+        <v>6.6</v>
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>Aging</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>05-08-2026</t>
         </is>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>07-08-2026</t>
+          <t>15-09-2026</t>
         </is>
       </c>
       <c r="AK11" t="n">
+        <v>41</v>
+      </c>
+      <c r="AL11" t="n">
         <v>43</v>
       </c>
-      <c r="AL11" t="n">
-        <v>84</v>
-      </c>
       <c r="AM11" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="AN11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AP11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AQ11" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="AR11" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="AS11" t="n">
-        <v>0</v>
+        <v>789002</v>
       </c>
       <c r="AT11" t="n">
-        <v>0</v>
+        <v>1412746</v>
       </c>
       <c r="AU11" t="n">
-        <v>0</v>
+        <v>5992468</v>
       </c>
       <c r="AV11" t="n">
-        <v>586966134</v>
+        <v>19457263</v>
       </c>
       <c r="AW11" t="n">
-        <v>595794044</v>
+        <v>19457263</v>
       </c>
       <c r="AX11" t="n">
-        <v>0</v>
+        <v>789002</v>
       </c>
       <c r="AY11" t="n">
-        <v>0</v>
+        <v>5992468</v>
       </c>
       <c r="AZ11" t="n">
         <v>1</v>
@@ -2573,7 +2571,7 @@
         <v>0</v>
       </c>
       <c r="BB11" t="n">
-        <v>0</v>
+        <v>0.1317</v>
       </c>
     </row>
     <row r="12">
@@ -2631,13 +2629,13 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.263</v>
+        <v>0.26</v>
       </c>
       <c r="Q12" t="n">
-        <v>875</v>
+        <v>886</v>
       </c>
       <c r="R12" t="n">
-        <v>8.6</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="S12" t="n">
         <v>7</v>
@@ -2813,13 +2811,13 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.047</v>
+        <v>0.048</v>
       </c>
       <c r="Q13" t="n">
-        <v>15314</v>
+        <v>15069</v>
       </c>
       <c r="R13" t="n">
-        <v>39</v>
+        <v>38.4</v>
       </c>
       <c r="S13" t="n">
         <v>83</v>
@@ -2943,16 +2941,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OBCL</t>
+          <t>ALEMBICLTD</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OBCL LIMITED</t>
+          <t>Alembic Limited</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2960,155 +2958,157 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G14" t="n">
+        <v>25</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>98.95</v>
+      </c>
+      <c r="J14" t="n">
+        <v>91.7</v>
+      </c>
+      <c r="K14" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="L14" t="n">
+        <v>70.88</v>
+      </c>
+      <c r="M14" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="N14" t="n">
         <v>5</v>
       </c>
-      <c r="G14" t="n">
-        <v>21</v>
-      </c>
-      <c r="H14" t="n">
-        <v>-1</v>
-      </c>
-      <c r="I14" t="n">
-        <v>56.98</v>
-      </c>
-      <c r="J14" t="n">
-        <v>53.45</v>
-      </c>
-      <c r="K14" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="L14" t="n">
-        <v>67.23</v>
-      </c>
-      <c r="M14" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="N14" t="n">
-        <v>11</v>
-      </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>15-09-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>1.625</v>
+        <v>0.322</v>
       </c>
       <c r="Q14" t="n">
-        <v>120</v>
-      </c>
-      <c r="R14" t="inlineStr"/>
+        <v>2638</v>
+      </c>
+      <c r="R14" t="n">
+        <v>21.6</v>
+      </c>
       <c r="S14" t="n">
+        <v>8</v>
+      </c>
+      <c r="T14" t="n">
+        <v>14</v>
+      </c>
+      <c r="U14" t="n">
+        <v>-14</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="W14" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Y14" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>93.37</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>92.28</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>91.7739742726077</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>17-08-2026</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>02-09-2026</t>
+        </is>
+      </c>
+      <c r="AK14" t="n">
+        <v>16</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>31</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>15</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>5</v>
+      </c>
+      <c r="AQ14" t="n">
         <v>6</v>
       </c>
-      <c r="T14" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="U14" t="n">
-        <v>-3779</v>
-      </c>
-      <c r="V14" t="n">
-        <v>-0.05</v>
-      </c>
-      <c r="W14" t="n">
-        <v>-1.26</v>
-      </c>
-      <c r="X14" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="Y14" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>54.13</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>55.15</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>53.44741172107844</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="AF14" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
-      <c r="AG14" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AH14" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AI14" t="inlineStr">
-        <is>
-          <t>05-08-2026</t>
-        </is>
-      </c>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
-      </c>
-      <c r="AK14" t="n">
-        <v>41</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>43</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO14" t="n">
-        <v>3</v>
-      </c>
-      <c r="AP14" t="n">
+      <c r="AR14" t="n">
         <v>6</v>
       </c>
-      <c r="AQ14" t="n">
-        <v>11</v>
-      </c>
-      <c r="AR14" t="n">
-        <v>11</v>
-      </c>
       <c r="AS14" t="n">
-        <v>789002</v>
+        <v>0</v>
       </c>
       <c r="AT14" t="n">
-        <v>1412746</v>
+        <v>0</v>
       </c>
       <c r="AU14" t="n">
-        <v>5992468</v>
+        <v>45956128</v>
       </c>
       <c r="AV14" t="n">
-        <v>19457263</v>
+        <v>85826103</v>
       </c>
       <c r="AW14" t="n">
-        <v>19457263</v>
+        <v>85826103</v>
       </c>
       <c r="AX14" t="n">
-        <v>789002</v>
+        <v>0</v>
       </c>
       <c r="AY14" t="n">
-        <v>5992468</v>
+        <v>45956128</v>
       </c>
       <c r="AZ14" t="n">
         <v>1</v>
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="BB14" t="n">
-        <v>0.1317</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3175,13 +3175,13 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.152</v>
+        <v>0.148</v>
       </c>
       <c r="Q15" t="n">
-        <v>728</v>
+        <v>748</v>
       </c>
       <c r="R15" t="n">
-        <v>60.8</v>
+        <v>62.5</v>
       </c>
       <c r="S15" t="n">
         <v>3</v>
@@ -3305,16 +3305,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -3322,91 +3322,91 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G16" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H16" t="n">
         <v>-1</v>
       </c>
       <c r="I16" t="n">
-        <v>190.06</v>
+        <v>602.05</v>
       </c>
       <c r="J16" t="n">
-        <v>170.45</v>
+        <v>616.75</v>
       </c>
       <c r="K16" t="n">
-        <v>11.5</v>
+        <v>-2.4</v>
       </c>
       <c r="L16" t="n">
-        <v>67.54000000000001</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="M16" t="n">
-        <v>0.26</v>
+        <v>4.4</v>
       </c>
       <c r="N16" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>0.102</v>
+        <v>0.383</v>
       </c>
       <c r="Q16" t="n">
-        <v>256</v>
+        <v>1148</v>
       </c>
       <c r="R16" t="n">
-        <v>27.4</v>
+        <v>58.5</v>
       </c>
       <c r="S16" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="T16" t="n">
-        <v>1.87</v>
+        <v>-0.11</v>
       </c>
       <c r="U16" t="n">
-        <v>-31</v>
+        <v>23</v>
       </c>
       <c r="V16" t="n">
-        <v>3.36</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="W16" t="n">
-        <v>4.96</v>
+        <v>1.58</v>
       </c>
       <c r="X16" t="n">
         <v>0</v>
       </c>
       <c r="Y16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z16" t="n">
-        <v>2.97</v>
+        <v>-110</v>
       </c>
       <c r="AA16" t="n">
-        <v>179.59</v>
+        <v>578.13</v>
       </c>
       <c r="AB16" t="n">
-        <v>162.67</v>
+        <v>513.73</v>
       </c>
       <c r="AC16" t="n">
-        <v>32.7</v>
+        <v>24.3</v>
       </c>
       <c r="AD16" t="n">
-        <v>170.4518641810919</v>
+        <v>616.7485587645351</v>
       </c>
       <c r="AE16" t="n">
-        <v>11.5</v>
+        <v>-2.4</v>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
@@ -3416,63 +3416,63 @@
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AI16" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>15-06-2026</t>
         </is>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="AL16" t="n">
-        <v>14</v>
+        <v>94</v>
       </c>
       <c r="AM16" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AN16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AP16" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="AQ16" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="AR16" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="AS16" t="n">
-        <v>0</v>
+        <v>938665</v>
       </c>
       <c r="AT16" t="n">
-        <v>5120374</v>
+        <v>2486819</v>
       </c>
       <c r="AU16" t="n">
-        <v>5120374</v>
+        <v>19027191</v>
       </c>
       <c r="AV16" t="n">
-        <v>5120374</v>
+        <v>21768420</v>
       </c>
       <c r="AW16" t="n">
-        <v>5120374</v>
+        <v>30053500</v>
       </c>
       <c r="AX16" t="n">
-        <v>0</v>
+        <v>938665</v>
       </c>
       <c r="AY16" t="n">
-        <v>5120374</v>
+        <v>19027191</v>
       </c>
       <c r="AZ16" t="n">
         <v>2</v>
@@ -3481,18 +3481,18 @@
         <v>0</v>
       </c>
       <c r="BB16" t="n">
-        <v>0</v>
+        <v>0.0493</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>PLASTIBLEN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>PLASTIBLENDS INDIA LIMITED</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -3504,181 +3504,181 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F17" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G17" t="n">
         <v>17</v>
       </c>
       <c r="H17" t="n">
-        <v>-1</v>
+        <v>-10</v>
       </c>
       <c r="I17" t="n">
-        <v>602.05</v>
+        <v>182.75</v>
       </c>
       <c r="J17" t="n">
-        <v>616.75</v>
+        <v>175.18</v>
       </c>
       <c r="K17" t="n">
-        <v>-2.4</v>
+        <v>4.3</v>
       </c>
       <c r="L17" t="n">
-        <v>64.68000000000001</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="M17" t="n">
-        <v>4.4</v>
+        <v>13.93</v>
       </c>
       <c r="N17" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.396</v>
+        <v>2.872</v>
       </c>
       <c r="Q17" t="n">
-        <v>1111</v>
+        <v>485</v>
       </c>
       <c r="R17" t="n">
-        <v>56.6</v>
+        <v>11.4</v>
       </c>
       <c r="S17" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="T17" t="n">
-        <v>-0.11</v>
+        <v>22</v>
       </c>
       <c r="U17" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="V17" t="n">
-        <v>-0.07000000000000001</v>
+        <v>5.75</v>
       </c>
       <c r="W17" t="n">
-        <v>1.58</v>
+        <v>10.7</v>
       </c>
       <c r="X17" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="Y17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z17" t="n">
-        <v>-110</v>
+        <v>10</v>
       </c>
       <c r="AA17" t="n">
-        <v>578.13</v>
+        <v>191.11</v>
       </c>
       <c r="AB17" t="n">
-        <v>513.73</v>
+        <v>166.71</v>
       </c>
       <c r="AC17" t="n">
-        <v>24.3</v>
+        <v>32.1</v>
       </c>
       <c r="AD17" t="n">
-        <v>616.7485587645351</v>
+        <v>175.1818845863716</v>
       </c>
       <c r="AE17" t="n">
-        <v>-2.4</v>
+        <v>4.3</v>
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Stale</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Stale Accumulation</t>
         </is>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>19-06-2026</t>
         </is>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="AK17" t="n">
-        <v>88</v>
+        <v>6</v>
       </c>
       <c r="AL17" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AM17" t="n">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="AN17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AP17" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="AQ17" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="AS17" t="n">
-        <v>938665</v>
+        <v>0</v>
       </c>
       <c r="AT17" t="n">
-        <v>2486819</v>
+        <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>19027191</v>
+        <v>0</v>
       </c>
       <c r="AV17" t="n">
-        <v>21768420</v>
+        <v>0</v>
       </c>
       <c r="AW17" t="n">
-        <v>30053500</v>
+        <v>79549544</v>
       </c>
       <c r="AX17" t="n">
-        <v>938665</v>
+        <v>0</v>
       </c>
       <c r="AY17" t="n">
-        <v>19027191</v>
+        <v>0</v>
       </c>
       <c r="AZ17" t="n">
         <v>2</v>
       </c>
       <c r="BA17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BB17" t="n">
-        <v>0.0493</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PLASTIBLEN</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PLASTIBLENDS INDIA LIMITED</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -3686,163 +3686,163 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G18" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H18" t="n">
-        <v>-10</v>
+        <v>-1</v>
       </c>
       <c r="I18" t="n">
-        <v>182.75</v>
+        <v>190.06</v>
       </c>
       <c r="J18" t="n">
-        <v>175.18</v>
+        <v>170.45</v>
       </c>
       <c r="K18" t="n">
-        <v>4.3</v>
+        <v>11.5</v>
       </c>
       <c r="L18" t="n">
-        <v>64.20999999999999</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="M18" t="n">
-        <v>13.93</v>
+        <v>0.26</v>
       </c>
       <c r="N18" t="n">
+        <v>2</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>03-09-2026</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>270</v>
+      </c>
+      <c r="R18" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="S18" t="n">
+        <v>24</v>
+      </c>
+      <c r="T18" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="U18" t="n">
+        <v>-31</v>
+      </c>
+      <c r="V18" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="W18" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="X18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>179.59</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>162.67</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>170.4518641810919</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>Mature — Wait for Pullback</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>03-09-2026</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>03-09-2026</t>
+        </is>
+      </c>
+      <c r="AK18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>14</v>
+      </c>
+      <c r="AM18" t="n">
+        <v>14</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO18" t="n">
         <v>4</v>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>25-06-2026</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>2.933</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>475</v>
-      </c>
-      <c r="R18" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="S18" t="n">
-        <v>5</v>
-      </c>
-      <c r="T18" t="n">
-        <v>22</v>
-      </c>
-      <c r="U18" t="n">
-        <v>36</v>
-      </c>
-      <c r="V18" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="W18" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="X18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="Y18" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA18" t="n">
-        <v>191.11</v>
-      </c>
-      <c r="AB18" t="n">
-        <v>166.71</v>
-      </c>
-      <c r="AC18" t="n">
-        <v>32.1</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>175.1818845863716</v>
-      </c>
-      <c r="AE18" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="AF18" t="inlineStr">
-        <is>
-          <t>Stale</t>
-        </is>
-      </c>
-      <c r="AG18" t="inlineStr">
-        <is>
-          <t>Stale Accumulation</t>
-        </is>
-      </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>Late — Poor Entry</t>
-        </is>
-      </c>
-      <c r="AI18" t="inlineStr">
-        <is>
-          <t>19-06-2026</t>
-        </is>
-      </c>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>25-06-2026</t>
-        </is>
-      </c>
-      <c r="AK18" t="n">
-        <v>6</v>
-      </c>
-      <c r="AL18" t="n">
-        <v>90</v>
-      </c>
-      <c r="AM18" t="n">
-        <v>84</v>
-      </c>
-      <c r="AN18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO18" t="n">
-        <v>0</v>
-      </c>
       <c r="AP18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AQ18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AR18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AS18" t="n">
         <v>0</v>
       </c>
       <c r="AT18" t="n">
-        <v>0</v>
+        <v>5120374</v>
       </c>
       <c r="AU18" t="n">
-        <v>0</v>
+        <v>5120374</v>
       </c>
       <c r="AV18" t="n">
-        <v>0</v>
+        <v>5120374</v>
       </c>
       <c r="AW18" t="n">
-        <v>79549544</v>
+        <v>5120374</v>
       </c>
       <c r="AX18" t="n">
         <v>0</v>
       </c>
       <c r="AY18" t="n">
-        <v>0</v>
+        <v>5120374</v>
       </c>
       <c r="AZ18" t="n">
         <v>2</v>
       </c>
       <c r="BA18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BB18" t="n">
         <v>0</v>
@@ -3903,13 +3903,13 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>0.111</v>
+        <v>0.11</v>
       </c>
       <c r="Q19" t="n">
-        <v>1575</v>
+        <v>1584</v>
       </c>
       <c r="R19" t="n">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="S19" t="n">
         <v>581</v>
@@ -4083,13 +4083,13 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.333</v>
+        <v>0.331</v>
       </c>
       <c r="Q20" t="n">
-        <v>3828</v>
+        <v>3858</v>
       </c>
       <c r="R20" t="n">
-        <v>86.2</v>
+        <v>86.8</v>
       </c>
       <c r="S20" t="n">
         <v>42</v>
@@ -4265,13 +4265,13 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>0.083</v>
+        <v>0.079</v>
       </c>
       <c r="Q21" t="n">
-        <v>410</v>
+        <v>431</v>
       </c>
       <c r="R21" t="n">
-        <v>12.1</v>
+        <v>12.7</v>
       </c>
       <c r="S21" t="n">
         <v>-8</v>
@@ -4447,13 +4447,13 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>1.106</v>
+        <v>1.077</v>
       </c>
       <c r="Q22" t="n">
-        <v>9285</v>
+        <v>9536</v>
       </c>
       <c r="R22" t="n">
-        <v>12.3</v>
+        <v>12.6</v>
       </c>
       <c r="S22" t="n">
         <v>-12</v>
@@ -4629,13 +4629,13 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.136</v>
+        <v>0.137</v>
       </c>
       <c r="Q23" t="n">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="R23" t="n">
-        <v>5.93</v>
+        <v>5.91</v>
       </c>
       <c r="S23" t="n">
         <v>118</v>
@@ -4807,13 +4807,13 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>0.198</v>
+        <v>0.196</v>
       </c>
       <c r="Q24" t="n">
-        <v>865</v>
+        <v>873</v>
       </c>
       <c r="R24" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="S24" t="n">
         <v>19</v>
@@ -4937,12 +4937,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KABRAEXTRU</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KABRA EXTRUSION TECHNIK LIMITED</t>
+          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -4954,177 +4954,173 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F25" t="n">
         <v>8</v>
       </c>
       <c r="G25" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="H25" t="n">
-        <v>-11</v>
+        <v>-1</v>
       </c>
       <c r="I25" t="n">
-        <v>628.1</v>
+        <v>13.06</v>
       </c>
       <c r="J25" t="n">
-        <v>240.47</v>
+        <v>12.87</v>
       </c>
       <c r="K25" t="n">
-        <v>161.2</v>
+        <v>1.5</v>
       </c>
       <c r="L25" t="n">
-        <v>60.24</v>
+        <v>69.12</v>
       </c>
       <c r="M25" t="n">
-        <v>13.64</v>
+        <v>2.28</v>
       </c>
       <c r="N25" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>0.621</v>
+        <v>0.651</v>
       </c>
       <c r="Q25" t="n">
-        <v>2197</v>
+        <v>350</v>
       </c>
       <c r="R25" t="n">
-        <v>650</v>
+        <v>1131</v>
       </c>
       <c r="S25" t="n">
+        <v>-61</v>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="n">
+        <v>-98</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="W25" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="Y25" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="n">
+        <v>11.83</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>12.83008398969399</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>10-08-2026</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>16-09-2026</t>
+        </is>
+      </c>
+      <c r="AK25" t="n">
+        <v>37</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>38</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN25" t="n">
         <v>3</v>
       </c>
-      <c r="T25" t="n">
-        <v>6.76</v>
-      </c>
-      <c r="U25" t="n">
-        <v>-81</v>
-      </c>
-      <c r="V25" t="n">
-        <v>-0.35</v>
-      </c>
-      <c r="W25" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="X25" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="Y25" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>5.43</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>482.84</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>294.93</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>172.4</v>
-      </c>
-      <c r="AD25" t="n">
-        <v>240.4691214206156</v>
-      </c>
-      <c r="AE25" t="n">
-        <v>161.2</v>
-      </c>
-      <c r="AF25" t="inlineStr">
-        <is>
-          <t>Stale</t>
-        </is>
-      </c>
-      <c r="AG25" t="inlineStr">
-        <is>
-          <t>Stale Accumulation</t>
-        </is>
-      </c>
-      <c r="AH25" t="inlineStr">
-        <is>
-          <t>Late — Poor Entry</t>
-        </is>
-      </c>
-      <c r="AI25" t="inlineStr">
-        <is>
-          <t>19-06-2026</t>
-        </is>
-      </c>
-      <c r="AJ25" t="inlineStr">
-        <is>
-          <t>25-06-2026</t>
-        </is>
-      </c>
-      <c r="AK25" t="n">
-        <v>6</v>
-      </c>
-      <c r="AL25" t="n">
-        <v>90</v>
-      </c>
-      <c r="AM25" t="n">
-        <v>84</v>
-      </c>
-      <c r="AN25" t="n">
-        <v>0</v>
-      </c>
       <c r="AO25" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AP25" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="AQ25" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AR25" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="AS25" t="n">
-        <v>0</v>
+        <v>3692319</v>
       </c>
       <c r="AT25" t="n">
-        <v>0</v>
+        <v>8083771</v>
       </c>
       <c r="AU25" t="n">
-        <v>0</v>
+        <v>14595510</v>
       </c>
       <c r="AV25" t="n">
-        <v>0</v>
+        <v>23419304</v>
       </c>
       <c r="AW25" t="n">
-        <v>76695745</v>
+        <v>23419304</v>
       </c>
       <c r="AX25" t="n">
-        <v>0</v>
+        <v>3692319</v>
       </c>
       <c r="AY25" t="n">
-        <v>0</v>
+        <v>14595510</v>
       </c>
       <c r="AZ25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BA25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB25" t="n">
-        <v>0</v>
+        <v>0.253</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>KABRAEXTRU</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
+          <t>KABRA EXTRUSION TECHNIK LIMITED</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -5136,163 +5132,163 @@
         </is>
       </c>
       <c r="E26" t="n">
+        <v>15</v>
+      </c>
+      <c r="F26" t="n">
+        <v>8</v>
+      </c>
+      <c r="G26" t="n">
+        <v>25</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-11</v>
+      </c>
+      <c r="I26" t="n">
+        <v>628.1</v>
+      </c>
+      <c r="J26" t="n">
+        <v>240.47</v>
+      </c>
+      <c r="K26" t="n">
+        <v>161.2</v>
+      </c>
+      <c r="L26" t="n">
+        <v>60.24</v>
+      </c>
+      <c r="M26" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="N26" t="n">
         <v>6</v>
       </c>
-      <c r="F26" t="n">
-        <v>26</v>
-      </c>
-      <c r="G26" t="n">
-        <v>5</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>153.05</v>
-      </c>
-      <c r="J26" t="n">
-        <v>171.84</v>
-      </c>
-      <c r="K26" t="n">
-        <v>-10.9</v>
-      </c>
-      <c r="L26" t="n">
-        <v>74.59</v>
-      </c>
-      <c r="M26" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="N26" t="n">
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>0.606</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>2249</v>
+      </c>
+      <c r="R26" t="n">
+        <v>665</v>
+      </c>
+      <c r="S26" t="n">
+        <v>3</v>
+      </c>
+      <c r="T26" t="n">
+        <v>6.76</v>
+      </c>
+      <c r="U26" t="n">
+        <v>-81</v>
+      </c>
+      <c r="V26" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="W26" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="X26" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="Y26" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>482.84</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>294.93</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>172.4</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>240.4691214206156</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>161.2</v>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>Stale</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>Stale Accumulation</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>Late — Poor Entry</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>19-06-2026</t>
+        </is>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="AK26" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>90</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>84</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR26" t="n">
         <v>4</v>
       </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>09-09-2026</t>
-        </is>
-      </c>
-      <c r="P26" t="n">
-        <v>0.057</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>1941</v>
-      </c>
-      <c r="R26" t="n">
-        <v>44.6</v>
-      </c>
-      <c r="S26" t="n">
-        <v>20</v>
-      </c>
-      <c r="T26" t="n">
-        <v>17</v>
-      </c>
-      <c r="U26" t="n">
-        <v>83</v>
-      </c>
-      <c r="V26" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="W26" t="n">
-        <v>30.3</v>
-      </c>
-      <c r="X26" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Y26" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z26" t="n">
-        <v>23</v>
-      </c>
-      <c r="AA26" t="n">
-        <v>187</v>
-      </c>
-      <c r="AB26" t="n">
-        <v>517.98</v>
-      </c>
-      <c r="AC26" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="AD26" t="n">
-        <v>170.7900804020101</v>
-      </c>
-      <c r="AE26" t="n">
-        <v>-10.4</v>
-      </c>
-      <c r="AF26" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="AG26" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AH26" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AI26" t="inlineStr">
-        <is>
-          <t>25-08-2026</t>
-        </is>
-      </c>
-      <c r="AJ26" t="inlineStr">
-        <is>
-          <t>09-09-2026</t>
-        </is>
-      </c>
-      <c r="AK26" t="n">
-        <v>15</v>
-      </c>
-      <c r="AL26" t="n">
-        <v>23</v>
-      </c>
-      <c r="AM26" t="n">
-        <v>8</v>
-      </c>
-      <c r="AN26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO26" t="n">
-        <v>7</v>
-      </c>
-      <c r="AP26" t="n">
-        <v>11</v>
-      </c>
-      <c r="AQ26" t="n">
-        <v>11</v>
-      </c>
-      <c r="AR26" t="n">
-        <v>11</v>
-      </c>
       <c r="AS26" t="n">
         <v>0</v>
       </c>
       <c r="AT26" t="n">
-        <v>24145516</v>
+        <v>0</v>
       </c>
       <c r="AU26" t="n">
-        <v>33987226</v>
+        <v>0</v>
       </c>
       <c r="AV26" t="n">
-        <v>33987226</v>
+        <v>0</v>
       </c>
       <c r="AW26" t="n">
-        <v>33987226</v>
+        <v>76695745</v>
       </c>
       <c r="AX26" t="n">
         <v>0</v>
       </c>
       <c r="AY26" t="n">
-        <v>33987226</v>
+        <v>0</v>
       </c>
       <c r="AZ26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BB26" t="n">
         <v>0</v>
@@ -5301,16 +5297,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GANESHCP</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
+          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -5318,160 +5314,160 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>163.07</v>
+        <v>153.05</v>
       </c>
       <c r="J27" t="n">
-        <v>189.45</v>
+        <v>171.84</v>
       </c>
       <c r="K27" t="n">
-        <v>-13.9</v>
+        <v>-10.9</v>
       </c>
       <c r="L27" t="n">
-        <v>64.08</v>
+        <v>74.59</v>
       </c>
       <c r="M27" t="n">
-        <v>3.4</v>
+        <v>1.1</v>
       </c>
       <c r="N27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>09-09-2026</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.516</v>
+        <v>0.057</v>
       </c>
       <c r="Q27" t="n">
-        <v>659</v>
+        <v>1941</v>
       </c>
       <c r="R27" t="n">
-        <v>14.5</v>
+        <v>44.6</v>
       </c>
       <c r="S27" t="n">
-        <v>-1</v>
+        <v>20</v>
       </c>
       <c r="T27" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="U27" t="n">
-        <v>45</v>
+        <v>83</v>
       </c>
       <c r="V27" t="n">
-        <v>3.1</v>
+        <v>0.8</v>
       </c>
       <c r="W27" t="n">
-        <v>19.3</v>
+        <v>30.3</v>
       </c>
       <c r="X27" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="Y27" t="b">
         <v>1</v>
       </c>
       <c r="Z27" t="n">
+        <v>23</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>187</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>517.98</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>170.7900804020101</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>-10.4</v>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>25-08-2026</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>09-09-2026</t>
+        </is>
+      </c>
+      <c r="AK27" t="n">
+        <v>15</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>23</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>8</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>7</v>
+      </c>
+      <c r="AP27" t="n">
         <v>11</v>
       </c>
-      <c r="AA27" t="n">
-        <v>170.63</v>
-      </c>
-      <c r="AB27" t="n">
-        <v>194.07</v>
-      </c>
-      <c r="AC27" t="n">
-        <v>-3.9</v>
-      </c>
-      <c r="AD27" t="n">
-        <v>189.4527941996654</v>
-      </c>
-      <c r="AE27" t="n">
-        <v>-13.9</v>
-      </c>
-      <c r="AF27" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="AG27" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AH27" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AI27" t="inlineStr">
-        <is>
-          <t>19-06-2026</t>
-        </is>
-      </c>
-      <c r="AJ27" t="inlineStr">
-        <is>
-          <t>02-09-2026</t>
-        </is>
-      </c>
-      <c r="AK27" t="n">
-        <v>75</v>
-      </c>
-      <c r="AL27" t="n">
-        <v>90</v>
-      </c>
-      <c r="AM27" t="n">
-        <v>15</v>
-      </c>
-      <c r="AN27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP27" t="n">
-        <v>2</v>
-      </c>
       <c r="AQ27" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="AR27" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="AS27" t="n">
         <v>0</v>
       </c>
       <c r="AT27" t="n">
-        <v>0</v>
+        <v>24145516</v>
       </c>
       <c r="AU27" t="n">
-        <v>8001009</v>
+        <v>33987226</v>
       </c>
       <c r="AV27" t="n">
-        <v>8001009</v>
+        <v>33987226</v>
       </c>
       <c r="AW27" t="n">
-        <v>23998951</v>
+        <v>33987226</v>
       </c>
       <c r="AX27" t="n">
         <v>0</v>
       </c>
       <c r="AY27" t="n">
-        <v>8001009</v>
+        <v>33987226</v>
       </c>
       <c r="AZ27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BA27" t="n">
         <v>0</v>
@@ -5483,12 +5479,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>GANESHCP</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -5500,162 +5496,166 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F28" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="G28" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>163.07</v>
+      </c>
+      <c r="J28" t="n">
+        <v>189.45</v>
+      </c>
+      <c r="K28" t="n">
+        <v>-13.9</v>
+      </c>
+      <c r="L28" t="n">
+        <v>64.08</v>
+      </c>
+      <c r="M28" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="N28" t="n">
+        <v>5</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>02-09-2026</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>0.501</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>679</v>
+      </c>
+      <c r="R28" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="S28" t="n">
         <v>-1</v>
       </c>
-      <c r="I28" t="n">
-        <v>13.06</v>
-      </c>
-      <c r="J28" t="n">
-        <v>12.86</v>
-      </c>
-      <c r="K28" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="L28" t="n">
-        <v>69.12</v>
-      </c>
-      <c r="M28" t="n">
-        <v>2.26</v>
-      </c>
-      <c r="N28" t="n">
-        <v>22</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>0.612</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>369</v>
-      </c>
-      <c r="R28" t="n">
-        <v>1189</v>
-      </c>
-      <c r="S28" t="n">
-        <v>-61</v>
-      </c>
-      <c r="T28" t="inlineStr"/>
+      <c r="T28" t="n">
+        <v>21</v>
+      </c>
       <c r="U28" t="n">
-        <v>-98</v>
+        <v>45</v>
       </c>
       <c r="V28" t="n">
-        <v>0.01</v>
+        <v>3.1</v>
       </c>
       <c r="W28" t="n">
-        <v>2.46</v>
+        <v>19.3</v>
       </c>
       <c r="X28" t="n">
-        <v>0.44</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Y28" t="b">
         <v>1</v>
       </c>
-      <c r="Z28" t="inlineStr"/>
+      <c r="Z28" t="n">
+        <v>11</v>
+      </c>
       <c r="AA28" t="n">
-        <v>11.83</v>
+        <v>170.63</v>
       </c>
       <c r="AB28" t="n">
-        <v>13.29</v>
+        <v>194.07</v>
       </c>
       <c r="AC28" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>189.4527941996654</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>-13.9</v>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>19-06-2026</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>02-09-2026</t>
+        </is>
+      </c>
+      <c r="AK28" t="n">
+        <v>75</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>90</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>15</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR28" t="n">
         <v>4</v>
       </c>
-      <c r="AD28" t="n">
-        <v>12.82446607045713</v>
-      </c>
-      <c r="AE28" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AF28" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
-      <c r="AG28" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AH28" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AI28" t="inlineStr">
-        <is>
-          <t>10-08-2026</t>
-        </is>
-      </c>
-      <c r="AJ28" t="inlineStr">
-        <is>
-          <t>15-09-2026</t>
-        </is>
-      </c>
-      <c r="AK28" t="n">
-        <v>36</v>
-      </c>
-      <c r="AL28" t="n">
-        <v>38</v>
-      </c>
-      <c r="AM28" t="n">
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>8001009</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>8001009</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>23998951</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>8001009</v>
+      </c>
+      <c r="AZ28" t="n">
         <v>2</v>
       </c>
-      <c r="AN28" t="n">
-        <v>2</v>
-      </c>
-      <c r="AO28" t="n">
-        <v>8</v>
-      </c>
-      <c r="AP28" t="n">
-        <v>18</v>
-      </c>
-      <c r="AQ28" t="n">
-        <v>23</v>
-      </c>
-      <c r="AR28" t="n">
-        <v>23</v>
-      </c>
-      <c r="AS28" t="n">
-        <v>3399131</v>
-      </c>
-      <c r="AT28" t="n">
-        <v>7790583</v>
-      </c>
-      <c r="AU28" t="n">
-        <v>14302322</v>
-      </c>
-      <c r="AV28" t="n">
-        <v>23126116</v>
-      </c>
-      <c r="AW28" t="n">
-        <v>23126116</v>
-      </c>
-      <c r="AX28" t="n">
-        <v>3399131</v>
-      </c>
-      <c r="AY28" t="n">
-        <v>14302322</v>
-      </c>
-      <c r="AZ28" t="n">
-        <v>1</v>
-      </c>
       <c r="BA28" t="n">
         <v>0</v>
       </c>
       <c r="BB28" t="n">
-        <v>0.2377</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -5716,10 +5716,10 @@
         <v>0.045</v>
       </c>
       <c r="Q29" t="n">
-        <v>925</v>
+        <v>941</v>
       </c>
       <c r="R29" t="n">
-        <v>98.90000000000001</v>
+        <v>101</v>
       </c>
       <c r="S29" t="n">
         <v>15</v>
@@ -5895,13 +5895,13 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.214</v>
+        <v>0.21</v>
       </c>
       <c r="Q30" t="n">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="R30" t="n">
-        <v>24.3</v>
+        <v>24.8</v>
       </c>
       <c r="S30" t="n">
         <v>12</v>
@@ -6077,13 +6077,13 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>0.039</v>
+        <v>0.038</v>
       </c>
       <c r="Q31" t="n">
-        <v>3421</v>
+        <v>3484</v>
       </c>
       <c r="R31" t="n">
-        <v>20.3</v>
+        <v>20.7</v>
       </c>
       <c r="S31" t="n">
         <v>-4</v>
@@ -6262,10 +6262,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="Q32" t="n">
-        <v>52254</v>
+        <v>52359</v>
       </c>
       <c r="R32" t="n">
-        <v>44.2</v>
+        <v>44.4</v>
       </c>
       <c r="S32" t="n">
         <v>5</v>
@@ -6441,13 +6441,13 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>0.431</v>
+        <v>0.424</v>
       </c>
       <c r="Q33" t="n">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="R33" t="n">
-        <v>37</v>
+        <v>37.7</v>
       </c>
       <c r="S33" t="n">
         <v>21</v>
@@ -6626,10 +6626,10 @@
         <v>0.052</v>
       </c>
       <c r="Q34" t="n">
-        <v>5015</v>
+        <v>5028</v>
       </c>
       <c r="R34" t="n">
-        <v>32.7</v>
+        <v>32.8</v>
       </c>
       <c r="S34" t="n">
         <v>-25</v>
@@ -6805,13 +6805,13 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
       <c r="Q35" t="n">
-        <v>5446</v>
+        <v>5560</v>
       </c>
       <c r="R35" t="n">
-        <v>9.199999999999999</v>
+        <v>9.42</v>
       </c>
       <c r="S35" t="n">
         <v>43</v>
@@ -6987,13 +6987,13 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>0.035</v>
+        <v>0.034</v>
       </c>
       <c r="Q36" t="n">
-        <v>3134</v>
+        <v>3161</v>
       </c>
       <c r="R36" t="n">
-        <v>21.2</v>
+        <v>21.4</v>
       </c>
       <c r="S36" t="n">
         <v>17</v>
@@ -7169,13 +7169,13 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>0.475</v>
+        <v>0.473</v>
       </c>
       <c r="Q37" t="n">
-        <v>3625</v>
+        <v>3638</v>
       </c>
       <c r="R37" t="n">
-        <v>25.4</v>
+        <v>25.5</v>
       </c>
       <c r="S37" t="n">
         <v>2</v>
@@ -7351,10 +7351,10 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>0.028</v>
+        <v>0.027</v>
       </c>
       <c r="Q38" t="n">
-        <v>904</v>
+        <v>921</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="n">
@@ -7531,13 +7531,13 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>2.256</v>
+        <v>2.227</v>
       </c>
       <c r="Q39" t="n">
-        <v>24706</v>
+        <v>25030</v>
       </c>
       <c r="R39" t="n">
-        <v>31.2</v>
+        <v>31.7</v>
       </c>
       <c r="S39" t="n">
         <v>-2</v>
@@ -7716,10 +7716,10 @@
         <v>0.043</v>
       </c>
       <c r="Q40" t="n">
-        <v>1593</v>
+        <v>1600</v>
       </c>
       <c r="R40" t="n">
-        <v>20.8</v>
+        <v>20.9</v>
       </c>
       <c r="S40" t="n">
         <v>10</v>
@@ -7895,13 +7895,13 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0.098</v>
+        <v>0.099</v>
       </c>
       <c r="Q41" t="n">
-        <v>1513</v>
+        <v>1502</v>
       </c>
       <c r="R41" t="n">
-        <v>13.7</v>
+        <v>13.6</v>
       </c>
       <c r="S41" t="n">
         <v>6</v>
@@ -8077,13 +8077,13 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.175</v>
+        <v>0.166</v>
       </c>
       <c r="Q42" t="n">
-        <v>710</v>
+        <v>747</v>
       </c>
       <c r="R42" t="n">
-        <v>12.9</v>
+        <v>13.6</v>
       </c>
       <c r="S42" t="n">
         <v>185</v>
@@ -8257,13 +8257,13 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>0.21</v>
+        <v>0.208</v>
       </c>
       <c r="Q43" t="n">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="R43" t="n">
-        <v>25.4</v>
+        <v>25.7</v>
       </c>
       <c r="S43" t="n">
         <v>21</v>
@@ -8441,7 +8441,7 @@
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="n">
-        <v>69.59999999999999</v>
+        <v>69</v>
       </c>
       <c r="S44" t="n">
         <v>-1</v>
@@ -8617,13 +8617,13 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>0.042</v>
+        <v>0.041</v>
       </c>
       <c r="Q45" t="n">
-        <v>737</v>
+        <v>755</v>
       </c>
       <c r="R45" t="n">
-        <v>48.1</v>
+        <v>49.2</v>
       </c>
       <c r="S45" t="n">
         <v>7</v>
@@ -8799,13 +8799,13 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0.131</v>
+        <v>0.132</v>
       </c>
       <c r="Q46" t="n">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="R46" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="S46" t="n">
         <v>61</v>
@@ -8979,13 +8979,13 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.2</v>
+        <v>0.202</v>
       </c>
       <c r="Q47" t="n">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="R47" t="n">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="S47" t="n">
         <v>19</v>
@@ -9164,10 +9164,10 @@
         <v>0.039</v>
       </c>
       <c r="Q48" t="n">
-        <v>786</v>
+        <v>799</v>
       </c>
       <c r="R48" t="n">
-        <v>18.8</v>
+        <v>19.1</v>
       </c>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="n">
@@ -9517,13 +9517,13 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0.054</v>
+        <v>0.053</v>
       </c>
       <c r="Q50" t="n">
-        <v>8779</v>
+        <v>8925</v>
       </c>
       <c r="R50" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
       <c r="S50" t="n">
         <v>21</v>
@@ -9702,10 +9702,10 @@
         <v>0.008</v>
       </c>
       <c r="Q51" t="n">
-        <v>112516</v>
+        <v>115188</v>
       </c>
       <c r="R51" t="n">
-        <v>32.4</v>
+        <v>33.2</v>
       </c>
       <c r="S51" t="n">
         <v>18</v>
@@ -9881,13 +9881,13 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>0.222</v>
+        <v>0.221</v>
       </c>
       <c r="Q52" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="R52" t="n">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="S52" t="n">
         <v>16</v>
@@ -10066,10 +10066,10 @@
         <v>0.043</v>
       </c>
       <c r="Q53" t="n">
-        <v>1454</v>
+        <v>1427</v>
       </c>
       <c r="R53" t="n">
-        <v>18.4</v>
+        <v>18.1</v>
       </c>
       <c r="S53" t="n">
         <v>13</v>
@@ -10248,7 +10248,7 @@
         <v>0.135</v>
       </c>
       <c r="Q54" t="n">
-        <v>1700</v>
+        <v>1702</v>
       </c>
       <c r="R54" t="n">
         <v>30.7</v>
@@ -10427,13 +10427,13 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>0.051</v>
+        <v>0.049</v>
       </c>
       <c r="Q55" t="n">
-        <v>920</v>
+        <v>953</v>
       </c>
       <c r="R55" t="n">
-        <v>25</v>
+        <v>25.9</v>
       </c>
       <c r="S55" t="n">
         <v>9</v>
@@ -10909,70 +10909,70 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ALEMBICLTD</t>
+          <t>DIAMONDYD</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alembic Limited</t>
+          <t>Prataap Snacks Limited</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>98.95</v>
+        <v>1102.2</v>
       </c>
       <c r="D10" t="n">
-        <v>91.7</v>
+        <v>1173.96</v>
       </c>
       <c r="E10" t="n">
-        <v>7.9</v>
+        <v>-6.1</v>
       </c>
       <c r="F10" t="n">
-        <v>70.88</v>
+        <v>69.75</v>
       </c>
       <c r="G10" t="n">
-        <v>8.49</v>
+        <v>59.58</v>
       </c>
       <c r="H10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>07-08-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DIAMONDYD</t>
+          <t>OBCL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Prataap Snacks Limited</t>
+          <t>OBCL LIMITED</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1102.2</v>
+        <v>56.98</v>
       </c>
       <c r="D11" t="n">
-        <v>1173.96</v>
+        <v>53.45</v>
       </c>
       <c r="E11" t="n">
-        <v>-6.1</v>
+        <v>6.6</v>
       </c>
       <c r="F11" t="n">
-        <v>69.75</v>
+        <v>67.23</v>
       </c>
       <c r="G11" t="n">
-        <v>59.58</v>
+        <v>1.95</v>
       </c>
       <c r="H11" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>07-08-2026</t>
+          <t>15-09-2026</t>
         </is>
       </c>
     </row>
@@ -11049,35 +11049,35 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OBCL</t>
+          <t>ALEMBICLTD</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OBCL LIMITED</t>
+          <t>Alembic Limited</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>56.98</v>
+        <v>98.95</v>
       </c>
       <c r="D14" t="n">
-        <v>53.45</v>
+        <v>91.7</v>
       </c>
       <c r="E14" t="n">
-        <v>6.6</v>
+        <v>7.9</v>
       </c>
       <c r="F14" t="n">
-        <v>67.23</v>
+        <v>70.88</v>
       </c>
       <c r="G14" t="n">
-        <v>1.95</v>
+        <v>8.49</v>
       </c>
       <c r="H14" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>15-09-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
     </row>
@@ -11119,105 +11119,105 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>190.06</v>
+        <v>602.05</v>
       </c>
       <c r="D16" t="n">
-        <v>170.45</v>
+        <v>616.75</v>
       </c>
       <c r="E16" t="n">
-        <v>11.5</v>
+        <v>-2.4</v>
       </c>
       <c r="F16" t="n">
-        <v>67.54000000000001</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>0.26</v>
+        <v>4.4</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>PLASTIBLEN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>PLASTIBLENDS INDIA LIMITED</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>602.05</v>
+        <v>182.75</v>
       </c>
       <c r="D17" t="n">
-        <v>616.75</v>
+        <v>175.18</v>
       </c>
       <c r="E17" t="n">
-        <v>-2.4</v>
+        <v>4.3</v>
       </c>
       <c r="F17" t="n">
-        <v>64.68000000000001</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>4.4</v>
+        <v>13.93</v>
       </c>
       <c r="H17" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PLASTIBLEN</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PLASTIBLENDS INDIA LIMITED</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>182.75</v>
+        <v>190.06</v>
       </c>
       <c r="D18" t="n">
-        <v>175.18</v>
+        <v>170.45</v>
       </c>
       <c r="E18" t="n">
-        <v>4.3</v>
+        <v>11.5</v>
       </c>
       <c r="F18" t="n">
-        <v>64.20999999999999</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="G18" t="n">
-        <v>13.93</v>
+        <v>0.26</v>
       </c>
       <c r="H18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
     </row>
@@ -11434,140 +11434,140 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KABRAEXTRU</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KABRA EXTRUSION TECHNIK LIMITED</t>
+          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>628.1</v>
+        <v>13.06</v>
       </c>
       <c r="D25" t="n">
-        <v>240.47</v>
+        <v>12.87</v>
       </c>
       <c r="E25" t="n">
-        <v>161.2</v>
+        <v>1.5</v>
       </c>
       <c r="F25" t="n">
-        <v>60.24</v>
+        <v>69.12</v>
       </c>
       <c r="G25" t="n">
-        <v>13.64</v>
+        <v>2.28</v>
       </c>
       <c r="H25" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>KABRAEXTRU</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
+          <t>KABRA EXTRUSION TECHNIK LIMITED</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>153.05</v>
+        <v>628.1</v>
       </c>
       <c r="D26" t="n">
-        <v>171.84</v>
+        <v>240.47</v>
       </c>
       <c r="E26" t="n">
-        <v>-10.9</v>
+        <v>161.2</v>
       </c>
       <c r="F26" t="n">
-        <v>74.59</v>
+        <v>60.24</v>
       </c>
       <c r="G26" t="n">
-        <v>1.1</v>
+        <v>13.64</v>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GANESHCP</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
+          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>163.07</v>
+        <v>153.05</v>
       </c>
       <c r="D27" t="n">
-        <v>189.45</v>
+        <v>171.84</v>
       </c>
       <c r="E27" t="n">
-        <v>-13.9</v>
+        <v>-10.9</v>
       </c>
       <c r="F27" t="n">
-        <v>64.08</v>
+        <v>74.59</v>
       </c>
       <c r="G27" t="n">
-        <v>3.4</v>
+        <v>1.1</v>
       </c>
       <c r="H27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>09-09-2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>GANESHCP</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>13.06</v>
+        <v>163.07</v>
       </c>
       <c r="D28" t="n">
-        <v>12.86</v>
+        <v>189.45</v>
       </c>
       <c r="E28" t="n">
-        <v>1.6</v>
+        <v>-13.9</v>
       </c>
       <c r="F28" t="n">
-        <v>69.12</v>
+        <v>64.08</v>
       </c>
       <c r="G28" t="n">
-        <v>2.26</v>
+        <v>3.4</v>
       </c>
       <c r="H28" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>15-09-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
     </row>

</xml_diff>